<commit_message>
progress: 71 village workbooks (sivaramans-llin 2026-10-10T20:40:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Kuruviagaram_13.427675_80.18543.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Kuruviagaram_13.427675_80.18543.xlsx
@@ -3290,6 +3290,11 @@
           <t>313</t>
         </is>
       </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -3297,6 +3302,11 @@
           <t>314</t>
         </is>
       </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -3304,6 +3314,11 @@
           <t>315</t>
         </is>
       </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -3311,6 +3326,11 @@
           <t>316</t>
         </is>
       </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -3318,6 +3338,11 @@
           <t>317</t>
         </is>
       </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -3325,6 +3350,11 @@
           <t>318</t>
         </is>
       </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -3332,6 +3362,11 @@
           <t>319</t>
         </is>
       </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -3339,6 +3374,11 @@
           <t>32</t>
         </is>
       </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -3346,6 +3386,11 @@
           <t>320</t>
         </is>
       </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -3353,6 +3398,11 @@
           <t>321</t>
         </is>
       </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -3360,6 +3410,11 @@
           <t>322</t>
         </is>
       </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -3367,6 +3422,11 @@
           <t>323</t>
         </is>
       </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -3374,6 +3434,11 @@
           <t>324</t>
         </is>
       </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -3381,6 +3446,11 @@
           <t>325</t>
         </is>
       </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -3388,6 +3458,11 @@
           <t>326</t>
         </is>
       </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -3395,6 +3470,11 @@
           <t>327</t>
         </is>
       </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -3402,6 +3482,11 @@
           <t>328</t>
         </is>
       </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -3409,6 +3494,11 @@
           <t>329</t>
         </is>
       </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -3416,6 +3506,11 @@
           <t>33</t>
         </is>
       </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -3423,6 +3518,11 @@
           <t>330</t>
         </is>
       </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4A, 4B, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -3430,6 +3530,11 @@
           <t>331</t>
         </is>
       </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -3437,6 +3542,11 @@
           <t>332</t>
         </is>
       </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -3444,6 +3554,11 @@
           <t>333</t>
         </is>
       </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -3451,6 +3566,11 @@
           <t>334</t>
         </is>
       </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -3458,6 +3578,11 @@
           <t>335</t>
         </is>
       </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -3465,6 +3590,11 @@
           <t>336</t>
         </is>
       </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -3472,6 +3602,11 @@
           <t>337</t>
         </is>
       </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -3479,6 +3614,11 @@
           <t>338</t>
         </is>
       </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -3486,6 +3626,11 @@
           <t>339</t>
         </is>
       </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -3493,6 +3638,11 @@
           <t>34</t>
         </is>
       </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>1A1, 1A1A, 1A1B, 1A2, 1B, 2A, 2B1, 2B2, 2B3</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -3500,6 +3650,11 @@
           <t>340</t>
         </is>
       </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -3507,6 +3662,11 @@
           <t>341</t>
         </is>
       </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -3514,6 +3674,11 @@
           <t>342</t>
         </is>
       </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -3521,6 +3686,11 @@
           <t>343</t>
         </is>
       </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -3528,6 +3698,11 @@
           <t>344</t>
         </is>
       </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -3535,6 +3710,11 @@
           <t>345</t>
         </is>
       </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -3542,6 +3722,11 @@
           <t>346</t>
         </is>
       </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -3549,6 +3734,11 @@
           <t>347</t>
         </is>
       </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -3556,6 +3746,11 @@
           <t>348</t>
         </is>
       </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -3563,6 +3758,11 @@
           <t>349</t>
         </is>
       </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -3570,6 +3770,11 @@
           <t>35</t>
         </is>
       </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -3577,6 +3782,11 @@
           <t>350</t>
         </is>
       </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -3584,6 +3794,11 @@
           <t>351</t>
         </is>
       </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -3591,6 +3806,11 @@
           <t>352</t>
         </is>
       </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -3598,6 +3818,11 @@
           <t>353</t>
         </is>
       </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3A, 3B, 4, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -3605,6 +3830,11 @@
           <t>354</t>
         </is>
       </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14A, 14B, 14C, 14D, 15, 16, 17, 18A, 18B, 18C, 19, 20, 21A, 21B, 21C1, 21C2, 21C3, 21C4, 21C5, 21C6, 21C7, 21C8, 21D, 21E, 22, 23A1, 23A2, 23B1, 23B2, 24, 2A, 2B, 2C, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -3612,6 +3842,11 @@
           <t>355</t>
         </is>
       </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -3619,6 +3854,11 @@
           <t>356</t>
         </is>
       </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -3626,6 +3866,11 @@
           <t>357</t>
         </is>
       </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -3633,6 +3878,11 @@
           <t>358</t>
         </is>
       </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -3640,6 +3890,11 @@
           <t>359</t>
         </is>
       </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -3647,6 +3902,11 @@
           <t>36</t>
         </is>
       </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -3654,6 +3914,11 @@
           <t>360</t>
         </is>
       </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>1, 1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -3661,6 +3926,11 @@
           <t>361</t>
         </is>
       </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -3668,6 +3938,11 @@
           <t>362</t>
         </is>
       </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -3675,6 +3950,11 @@
           <t>363</t>
         </is>
       </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -3682,6 +3962,11 @@
           <t>364</t>
         </is>
       </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -3689,6 +3974,11 @@
           <t>365</t>
         </is>
       </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -3696,6 +3986,11 @@
           <t>366</t>
         </is>
       </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -3703,6 +3998,11 @@
           <t>367</t>
         </is>
       </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B1, 3B2, 4, 5, 6, 7A, 7B, 8</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -3710,6 +4010,11 @@
           <t>368</t>
         </is>
       </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -3717,6 +4022,11 @@
           <t>369</t>
         </is>
       </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A1A, 2A2, 2B, 2C, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -3724,6 +4034,11 @@
           <t>37</t>
         </is>
       </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -3731,6 +4046,11 @@
           <t>370</t>
         </is>
       </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>1A, 1B1A, 1B2, 1B3, 1B4, 2A1, 2A2, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -3738,6 +4058,11 @@
           <t>371</t>
         </is>
       </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -3745,6 +4070,11 @@
           <t>372</t>
         </is>
       </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -3752,6 +4082,11 @@
           <t>373</t>
         </is>
       </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -3759,6 +4094,11 @@
           <t>374</t>
         </is>
       </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C, 3D, 3E</t>
+        </is>
+      </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -3766,6 +4106,11 @@
           <t>375</t>
         </is>
       </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -3773,6 +4118,11 @@
           <t>376</t>
         </is>
       </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -3780,6 +4130,11 @@
           <t>377</t>
         </is>
       </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -3787,6 +4142,11 @@
           <t>378</t>
         </is>
       </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -3794,6 +4154,11 @@
           <t>379</t>
         </is>
       </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -3801,6 +4166,11 @@
           <t>38</t>
         </is>
       </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -3808,6 +4178,11 @@
           <t>380</t>
         </is>
       </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3, 4A, 4B, 5, 6, 7A, 7B</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -3815,6 +4190,11 @@
           <t>381</t>
         </is>
       </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -3822,6 +4202,11 @@
           <t>382</t>
         </is>
       </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -3829,6 +4214,11 @@
           <t>383</t>
         </is>
       </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -3836,6 +4226,11 @@
           <t>384</t>
         </is>
       </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -3843,11 +4238,21 @@
           <t>385</t>
         </is>
       </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
           <t>386</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 71 village workbooks (sivaramans-llin 2026-10-10T20:50:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Kuruviagaram_13.427675_80.18543.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Kuruviagaram_13.427675_80.18543.xlsx
@@ -4262,6 +4262,11 @@
           <t>387</t>
         </is>
       </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -4269,6 +4274,11 @@
           <t>388</t>
         </is>
       </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1C, 1D1, 1D2, 2</t>
+        </is>
+      </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -4276,6 +4286,11 @@
           <t>389</t>
         </is>
       </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -4283,6 +4298,11 @@
           <t>39</t>
         </is>
       </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -4290,6 +4310,11 @@
           <t>390</t>
         </is>
       </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -4297,6 +4322,11 @@
           <t>391</t>
         </is>
       </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -4304,6 +4334,11 @@
           <t>392</t>
         </is>
       </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -4311,6 +4346,11 @@
           <t>393</t>
         </is>
       </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -4318,6 +4358,11 @@
           <t>394</t>
         </is>
       </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -4325,6 +4370,11 @@
           <t>395</t>
         </is>
       </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -4332,6 +4382,11 @@
           <t>396</t>
         </is>
       </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -4339,6 +4394,11 @@
           <t>397</t>
         </is>
       </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -4346,6 +4406,11 @@
           <t>398</t>
         </is>
       </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -4353,6 +4418,11 @@
           <t>399</t>
         </is>
       </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -4360,6 +4430,11 @@
           <t>4</t>
         </is>
       </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12, 13, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -4367,6 +4442,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -4374,6 +4454,11 @@
           <t>400</t>
         </is>
       </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
@@ -4381,6 +4466,11 @@
           <t>401</t>
         </is>
       </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5, 6A, 6B, 7</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -4388,6 +4478,11 @@
           <t>402</t>
         </is>
       </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2, 2C, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -4395,6 +4490,11 @@
           <t>403</t>
         </is>
       </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -4402,6 +4502,11 @@
           <t>406</t>
         </is>
       </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -4409,6 +4514,11 @@
           <t>407</t>
         </is>
       </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -4416,6 +4526,11 @@
           <t>41</t>
         </is>
       </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
@@ -4423,6 +4538,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
@@ -4430,6 +4550,11 @@
           <t>43</t>
         </is>
       </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -4437,6 +4562,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
@@ -4444,6 +4574,11 @@
           <t>45</t>
         </is>
       </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
@@ -4451,6 +4586,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2, 2B3, 2B4, 2B5, 2B6, 2B7</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -4458,6 +4598,11 @@
           <t>47</t>
         </is>
       </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -4465,6 +4610,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -4472,6 +4622,11 @@
           <t>49</t>
         </is>
       </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -4479,6 +4634,11 @@
           <t>5</t>
         </is>
       </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
@@ -4486,6 +4646,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
@@ -4493,6 +4658,11 @@
           <t>51</t>
         </is>
       </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -4500,6 +4670,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
@@ -4507,6 +4682,11 @@
           <t>53</t>
         </is>
       </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
@@ -4514,6 +4694,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -4521,6 +4706,11 @@
           <t>55</t>
         </is>
       </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -4528,6 +4718,11 @@
           <t>56</t>
         </is>
       </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -4535,6 +4730,11 @@
           <t>57</t>
         </is>
       </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B1, 5B2, 6A</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -4542,6 +4742,11 @@
           <t>58</t>
         </is>
       </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -4549,6 +4754,11 @@
           <t>59</t>
         </is>
       </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -4556,6 +4766,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -4563,6 +4778,11 @@
           <t>60</t>
         </is>
       </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -4570,6 +4790,11 @@
           <t>61</t>
         </is>
       </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2A, 2B, 2C, 3, 4, 5A, 5B1, 5B2, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -4577,6 +4802,11 @@
           <t>62</t>
         </is>
       </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -4584,6 +4814,11 @@
           <t>63</t>
         </is>
       </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -4591,6 +4826,11 @@
           <t>64</t>
         </is>
       </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
@@ -4598,6 +4838,11 @@
           <t>65</t>
         </is>
       </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B7B8B9B, 6, 7A, 8A, 9A</t>
+        </is>
+      </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
@@ -4605,6 +4850,11 @@
           <t>66</t>
         </is>
       </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
@@ -4612,6 +4862,11 @@
           <t>67</t>
         </is>
       </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
@@ -4619,6 +4874,11 @@
           <t>68</t>
         </is>
       </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
@@ -4626,6 +4886,11 @@
           <t>69</t>
         </is>
       </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
@@ -4633,6 +4898,11 @@
           <t>7</t>
         </is>
       </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
@@ -4640,6 +4910,11 @@
           <t>70</t>
         </is>
       </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
@@ -4647,6 +4922,11 @@
           <t>71</t>
         </is>
       </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
@@ -4654,6 +4934,11 @@
           <t>72</t>
         </is>
       </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
@@ -4661,6 +4946,11 @@
           <t>73</t>
         </is>
       </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
@@ -4668,6 +4958,11 @@
           <t>74</t>
         </is>
       </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
@@ -4675,6 +4970,11 @@
           <t>75</t>
         </is>
       </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
@@ -4682,6 +4982,11 @@
           <t>76</t>
         </is>
       </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
@@ -4689,6 +4994,11 @@
           <t>77</t>
         </is>
       </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
@@ -4696,6 +5006,11 @@
           <t>78</t>
         </is>
       </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
@@ -4703,6 +5018,11 @@
           <t>79</t>
         </is>
       </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
@@ -4710,6 +5030,11 @@
           <t>8</t>
         </is>
       </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
@@ -4717,6 +5042,11 @@
           <t>80</t>
         </is>
       </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B, 4A, 4B, 5A, 5B1, 5B2, 5B3, 5C, 5D, 5E, 5F, 5G, 5H, 6A, 6B, 6C, 6D, 6E, 6F, 6G, 7</t>
+        </is>
+      </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
@@ -4724,6 +5054,11 @@
           <t>81</t>
         </is>
       </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2A, 2B, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
@@ -4731,6 +5066,11 @@
           <t>82</t>
         </is>
       </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
@@ -4738,11 +5078,21 @@
           <t>83</t>
         </is>
       </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
           <t>84</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
         </is>
       </c>
     </row>

</xml_diff>